<commit_message>
modified wbs and added roles for 100% activity
</commit_message>
<xml_diff>
--- a/WBS - Contx.xlsx
+++ b/WBS - Contx.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mel\CodingProjects\capdocs-panic\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\Summer\capdocs-panic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD079F16-8208-4F19-8533-F7927D4429D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C087AF-80E5-4B41-AC84-0B658062585F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WBS" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="284">
   <si>
     <t>WBS Code</t>
   </si>
@@ -871,6 +871,9 @@
   </si>
   <si>
     <t>- This is a teaching example; adjust Dev count, durations, and start date to fit your own class project.</t>
+  </si>
+  <si>
+    <t>Ongoing</t>
   </si>
 </sst>
 </file>
@@ -1654,19 +1657,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K94"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="42.5546875" style="9" customWidth="1"/>
-    <col min="3" max="3" width="42.109375" style="9" customWidth="1"/>
-    <col min="4" max="4" width="12.21875" customWidth="1"/>
+    <col min="2" max="2" width="42.5703125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="42.140625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="15.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -1701,7 +1704,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>11</v>
       </c>
@@ -1722,7 +1725,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="87" t="s">
         <v>15</v>
       </c>
@@ -1757,7 +1760,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="87" t="s">
         <v>19</v>
       </c>
@@ -1792,7 +1795,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="87" t="s">
         <v>22</v>
       </c>
@@ -1827,7 +1830,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>25</v>
       </c>
@@ -1848,7 +1851,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
         <v>27</v>
       </c>
@@ -1883,7 +1886,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="68" t="s">
         <v>31</v>
       </c>
@@ -1918,7 +1921,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="68" t="s">
         <v>34</v>
       </c>
@@ -1953,7 +1956,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="68" t="s">
         <v>37</v>
       </c>
@@ -1988,7 +1991,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="68" t="s">
         <v>40</v>
       </c>
@@ -2023,7 +2026,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="68" t="s">
         <v>43</v>
       </c>
@@ -2058,7 +2061,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="38" t="s">
         <v>46</v>
       </c>
@@ -2093,7 +2096,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="43">
         <v>1.3</v>
       </c>
@@ -2128,7 +2131,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="80">
         <v>1.4</v>
       </c>
@@ -2163,7 +2166,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="43">
         <v>1.5</v>
       </c>
@@ -2198,7 +2201,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>57</v>
       </c>
@@ -2219,7 +2222,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="46" t="s">
         <v>59</v>
       </c>
@@ -2254,7 +2257,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="46" t="s">
         <v>62</v>
       </c>
@@ -2289,7 +2292,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="46" t="s">
         <v>65</v>
       </c>
@@ -2324,7 +2327,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="46" t="s">
         <v>68</v>
       </c>
@@ -2359,7 +2362,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="46" t="s">
         <v>71</v>
       </c>
@@ -2394,7 +2397,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
         <v>74</v>
       </c>
@@ -2415,7 +2418,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="46" t="s">
         <v>76</v>
       </c>
@@ -2450,7 +2453,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="46" t="s">
         <v>79</v>
       </c>
@@ -2485,7 +2488,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
         <v>82</v>
       </c>
@@ -2506,7 +2509,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="38" t="s">
         <v>84</v>
       </c>
@@ -2541,7 +2544,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="55" t="s">
         <v>87</v>
       </c>
@@ -2576,7 +2579,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="55" t="s">
         <v>91</v>
       </c>
@@ -2611,7 +2614,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="38" t="s">
         <v>94</v>
       </c>
@@ -2646,7 +2649,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
         <v>97</v>
       </c>
@@ -2667,7 +2670,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="61" t="s">
         <v>99</v>
       </c>
@@ -2702,7 +2705,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="87" t="s">
         <v>102</v>
       </c>
@@ -2737,7 +2740,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
         <v>106</v>
       </c>
@@ -2758,7 +2761,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="38" t="s">
         <v>108</v>
       </c>
@@ -2793,7 +2796,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="87" t="s">
         <v>111</v>
       </c>
@@ -2828,7 +2831,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="87" t="s">
         <v>114</v>
       </c>
@@ -2863,7 +2866,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
         <v>117</v>
       </c>
@@ -2884,7 +2887,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="38" t="s">
         <v>119</v>
       </c>
@@ -2919,7 +2922,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="60">
         <v>7.2</v>
       </c>
@@ -2954,7 +2957,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
         <v>124</v>
       </c>
@@ -2975,7 +2978,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="55" t="s">
         <v>126</v>
       </c>
@@ -3010,7 +3013,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="55" t="s">
         <v>129</v>
       </c>
@@ -3043,7 +3046,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="73" t="s">
         <v>131</v>
       </c>
@@ -3078,7 +3081,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="73" t="s">
         <v>134</v>
       </c>
@@ -3113,7 +3116,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="55" t="s">
         <v>137</v>
       </c>
@@ -3146,7 +3149,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="73" t="s">
         <v>139</v>
       </c>
@@ -3181,7 +3184,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="73" t="s">
         <v>142</v>
       </c>
@@ -3216,7 +3219,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="73" t="s">
         <v>145</v>
       </c>
@@ -3251,7 +3254,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="73" t="s">
         <v>148</v>
       </c>
@@ -3286,7 +3289,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="73" t="s">
         <v>151</v>
       </c>
@@ -3321,7 +3324,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="55" t="s">
         <v>154</v>
       </c>
@@ -3356,7 +3359,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="31" t="s">
         <v>157</v>
       </c>
@@ -3377,7 +3380,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="81" t="s">
         <v>159</v>
       </c>
@@ -3412,7 +3415,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="81" t="s">
         <v>162</v>
       </c>
@@ -3447,7 +3450,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A56" s="81" t="s">
         <v>165</v>
       </c>
@@ -3482,7 +3485,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="31" t="s">
         <v>168</v>
       </c>
@@ -3503,7 +3506,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="96" t="s">
         <v>170</v>
       </c>
@@ -3538,7 +3541,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="22" t="s">
         <v>173</v>
       </c>
@@ -3567,7 +3570,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
         <v>25</v>
       </c>
@@ -3588,7 +3591,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="43">
         <v>1.6</v>
       </c>
@@ -3617,7 +3620,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="43">
         <v>1.7</v>
       </c>
@@ -3643,10 +3646,10 @@
       <c r="I62" s="44"/>
       <c r="J62" s="44"/>
       <c r="K62" s="42" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="43">
         <v>1.8</v>
       </c>
@@ -3675,7 +3678,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="13" t="s">
         <v>97</v>
       </c>
@@ -3696,7 +3699,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="61" t="s">
         <v>184</v>
       </c>
@@ -3725,7 +3728,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="13" t="s">
         <v>117</v>
       </c>
@@ -3746,7 +3749,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A67" s="80">
         <v>7.3</v>
       </c>
@@ -3775,7 +3778,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="43">
         <v>7.4</v>
       </c>
@@ -3801,10 +3804,10 @@
       <c r="I68" s="44"/>
       <c r="J68" s="44"/>
       <c r="K68" s="42" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="28" t="s">
         <v>192</v>
       </c>
@@ -3815,7 +3818,7 @@
         <v>194</v>
       </c>
       <c r="D69" s="28" t="s">
-        <v>195</v>
+        <v>30</v>
       </c>
       <c r="E69" s="28"/>
       <c r="F69" s="28" t="s">
@@ -3830,10 +3833,10 @@
       <c r="I69" s="28"/>
       <c r="J69" s="28"/>
       <c r="K69" s="18" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="28" t="s">
         <v>196</v>
       </c>
@@ -3844,7 +3847,7 @@
         <v>198</v>
       </c>
       <c r="D70" s="28" t="s">
-        <v>195</v>
+        <v>53</v>
       </c>
       <c r="E70" s="28"/>
       <c r="F70" s="28" t="s">
@@ -3862,7 +3865,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="28" t="s">
         <v>199</v>
       </c>
@@ -3873,7 +3876,7 @@
         <v>201</v>
       </c>
       <c r="D71" s="28" t="s">
-        <v>195</v>
+        <v>90</v>
       </c>
       <c r="E71" s="28"/>
       <c r="F71" s="28" t="s">
@@ -3891,7 +3894,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="13" t="s">
         <v>124</v>
       </c>
@@ -3912,7 +3915,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="55" t="s">
         <v>203</v>
       </c>
@@ -3941,7 +3944,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="20">
         <v>8.6</v>
       </c>
@@ -3952,7 +3955,7 @@
         <v>207</v>
       </c>
       <c r="D74" s="28" t="s">
-        <v>195</v>
+        <v>90</v>
       </c>
       <c r="E74" s="28"/>
       <c r="F74" s="28" t="s">
@@ -3970,7 +3973,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="31" t="s">
         <v>208</v>
       </c>
@@ -3991,7 +3994,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A76" s="28" t="s">
         <v>210</v>
       </c>
@@ -4002,7 +4005,7 @@
         <v>212</v>
       </c>
       <c r="D76" s="28" t="s">
-        <v>195</v>
+        <v>90</v>
       </c>
       <c r="E76" s="28"/>
       <c r="F76" s="28" t="s">
@@ -4020,7 +4023,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A77" s="28" t="s">
         <v>213</v>
       </c>
@@ -4031,7 +4034,7 @@
         <v>215</v>
       </c>
       <c r="D77" s="28" t="s">
-        <v>195</v>
+        <v>30</v>
       </c>
       <c r="E77" s="28"/>
       <c r="F77" s="28" t="s">
@@ -4046,10 +4049,10 @@
       <c r="I77" s="28"/>
       <c r="J77" s="28"/>
       <c r="K77" s="18" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="28" t="s">
         <v>216</v>
       </c>
@@ -4060,7 +4063,7 @@
         <v>218</v>
       </c>
       <c r="D78" s="28" t="s">
-        <v>195</v>
+        <v>30</v>
       </c>
       <c r="E78" s="28"/>
       <c r="F78" s="28" t="s">
@@ -4078,7 +4081,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="86">
         <v>11</v>
       </c>
@@ -4099,7 +4102,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="28" t="s">
         <v>220</v>
       </c>
@@ -4110,7 +4113,7 @@
         <v>222</v>
       </c>
       <c r="D80" s="28" t="s">
-        <v>195</v>
+        <v>53</v>
       </c>
       <c r="E80" s="28"/>
       <c r="F80" s="28" t="s">
@@ -4128,7 +4131,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="28" t="s">
         <v>223</v>
       </c>
@@ -4139,7 +4142,7 @@
         <v>225</v>
       </c>
       <c r="D81" s="28" t="s">
-        <v>195</v>
+        <v>53</v>
       </c>
       <c r="E81" s="28"/>
       <c r="F81" s="28" t="s">
@@ -4157,7 +4160,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="28" t="s">
         <v>226</v>
       </c>
@@ -4168,7 +4171,7 @@
         <v>228</v>
       </c>
       <c r="D82" s="28" t="s">
-        <v>195</v>
+        <v>53</v>
       </c>
       <c r="E82" s="28"/>
       <c r="F82" s="28" t="s">
@@ -4186,7 +4189,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="28" t="s">
         <v>229</v>
       </c>
@@ -4197,7 +4200,7 @@
         <v>231</v>
       </c>
       <c r="D83" s="28" t="s">
-        <v>195</v>
+        <v>53</v>
       </c>
       <c r="E83" s="28"/>
       <c r="F83" s="28" t="s">
@@ -4215,7 +4218,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="31" t="s">
         <v>168</v>
       </c>
@@ -4236,7 +4239,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="85" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="28" t="s">
         <v>232</v>
       </c>
@@ -4265,7 +4268,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="86" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="28" t="s">
         <v>236</v>
       </c>
@@ -4294,7 +4297,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="31" t="s">
         <v>240</v>
       </c>
@@ -4315,7 +4318,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="88" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="28" t="s">
         <v>242</v>
       </c>
@@ -4326,7 +4329,7 @@
         <v>244</v>
       </c>
       <c r="D88" s="28" t="s">
-        <v>195</v>
+        <v>18</v>
       </c>
       <c r="E88" s="28"/>
       <c r="F88" s="28" t="s">
@@ -4344,7 +4347,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="28" t="s">
         <v>246</v>
       </c>
@@ -4355,7 +4358,7 @@
         <v>248</v>
       </c>
       <c r="D89" s="28" t="s">
-        <v>195</v>
+        <v>18</v>
       </c>
       <c r="E89" s="28"/>
       <c r="F89" s="28" t="s">
@@ -4373,7 +4376,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="28" t="s">
         <v>249</v>
       </c>
@@ -4384,7 +4387,7 @@
         <v>251</v>
       </c>
       <c r="D90" s="28" t="s">
-        <v>195</v>
+        <v>18</v>
       </c>
       <c r="E90" s="28"/>
       <c r="F90" s="28" t="s">
@@ -4402,7 +4405,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="31" t="s">
         <v>252</v>
       </c>
@@ -4423,7 +4426,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="28" t="s">
         <v>254</v>
       </c>
@@ -4434,7 +4437,7 @@
         <v>256</v>
       </c>
       <c r="D92" s="28" t="s">
-        <v>195</v>
+        <v>18</v>
       </c>
       <c r="E92" s="28"/>
       <c r="F92" s="28" t="s">
@@ -4452,7 +4455,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="28" t="s">
         <v>257</v>
       </c>
@@ -4463,7 +4466,7 @@
         <v>259</v>
       </c>
       <c r="D93" s="28" t="s">
-        <v>195</v>
+        <v>18</v>
       </c>
       <c r="E93" s="28"/>
       <c r="F93" s="28" t="s">
@@ -4481,7 +4484,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="94" spans="1:11" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="35" t="s">
         <v>260</v>
       </c>
@@ -4519,18 +4522,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>263</v>
       </c>
@@ -4538,7 +4541,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>265</v>
       </c>
@@ -4546,7 +4549,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>267</v>
       </c>
@@ -4554,7 +4557,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>269</v>
       </c>
@@ -4562,65 +4565,65 @@
         <v>270</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>282</v>
       </c>

</xml_diff>